<commit_message>
preserve custom point values
</commit_message>
<xml_diff>
--- a/frontend/public/templates/优才计划团队积分批量导入模板.xlsx
+++ b/frontend/public/templates/优才计划团队积分批量导入模板.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="团队积分导入" sheetId="1" r:id="R48ae559292e24645"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="Rb050cac239264572"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="下拉选项" sheetId="3" r:id="R69d42c7eaf6b438f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="团队积分导入" sheetId="1" r:id="Rb4dce583830f4c9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="R8a06276436d4486c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="下拉选项" sheetId="3" r:id="R29d6f6ee19c749e5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2696,31 +2696,28 @@
       <x:c r="H501" s="30"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="8">
-    <x:dataValidation type="list" sqref="A2:A501">
-      <x:formula1>'下拉选项'!$A$2:$A$50</x:formula1>
+  <x:dataValidations count="7">
+    <x:dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="A2:A200">
+      <x:formula1>'下拉选项'!$A$2:$A$4</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="B2:B501">
-      <x:formula1>'下拉选项'!$B$2:$B$50</x:formula1>
+    <x:dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B200">
+      <x:formula1>'下拉选项'!$B$2:$B$3</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C2:C501">
-      <x:formula1>'下拉选项'!$C$2:$C$50</x:formula1>
+    <x:dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C200">
+      <x:formula1>'下拉选项'!$C$2:$C$5</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="D2:D501">
-      <x:formula1>'下拉选项'!$D$2:$D$100</x:formula1>
+    <x:dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D200">
+      <x:formula1>'下拉选项'!$D$2:$D$11</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="E2:E501">
+    <x:dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E200">
       <x:formula1>'下拉选项'!$E$2:$E$6</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="G2:G501">
-      <x:formula1>'下拉选项'!$F$2:$F$9</x:formula1>
+    <x:dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I2:I200">
+      <x:formula1>'下拉选项'!$G$2:$G$7</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="date" operator="between" sqref="H2:H501">
+    <x:dataValidation type="date" operator="between" allowBlank="1" showErrorMessage="1" sqref="H2:H200">
       <x:formula1>2020-01-01</x:formula1>
       <x:formula2>2099-12-31</x:formula2>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="I2:I501">
-      <x:formula1>'下拉选项'!$G$2:$G$7</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2737,7 +2734,7 @@
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
       <x:c r="A1" s="50" t="str">
-        <x:v>优才计划团队积分批量导入模板</x:v>
+        <x:v>优才计划小组积分批量导入模板</x:v>
       </x:c>
       <x:c r="B1" s="50" t="str">
         <x:v>优才计划团队积分批量导入模板</x:v>
@@ -2776,7 +2773,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B5" s="49" t="str">
-        <x:v>回到“团队积分导入”工作表，从下拉列表选择年度、项目、阶段、小组、积分类别、积分值和数据来源。</x:v>
+        <x:v>回到“团队积分导入”工作表，从下拉列表选择年度、项目、阶段、小组、积分类别和数据来源；积分值直接填写任意非零整数。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
@@ -2792,7 +2789,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B7" s="49" t="str">
-        <x:v>线上案例沟通、线上案例输出会按获得日期自动排序计分：前2组20分、第3—4组15分、后续10分。</x:v>
+        <x:v>系统会完全按照“积分值”列记录小组积分，不会根据积分类别、获得日期或提交顺序自动改写分值。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
@@ -2808,7 +2805,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B9" s="49" t="str">
-        <x:v>每行代表一笔团队积分；请勿修改“团队积分导入”工作表的列名。</x:v>
+        <x:v>每行代表一笔小组积分；请勿修改“团队积分导入”工作表的列名。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
@@ -2816,7 +2813,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B10" s="49" t="str">
-        <x:v>完成后在管理端“团队积分”页面点击“Excel批量导入”，系统会先预览和检查错误。</x:v>
+        <x:v>完成后在管理端“小组积分”页面点击“Excel批量导入”，系统会先预览和检查错误。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2836,7 +2833,7 @@
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -2857,7 +2854,7 @@
         <x:v>积分类别</x:v>
       </x:c>
       <x:c r="F1" s="37" t="str">
-        <x:v>积分值</x:v>
+        <x:v>积分值示例（可自定义）</x:v>
       </x:c>
       <x:c r="G1" s="37" t="str">
         <x:v>数据来源</x:v>

</xml_diff>